<commit_message>
feat(day22): complete missing metrics, stranger test S10 and full indicators
</commit_message>
<xml_diff>
--- a/NguyenQuangHuy_Day22_model.xlsx
+++ b/NguyenQuangHuy_Day22_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAY22_Track1_2A202602421_NguyenQuangHuy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083E069F-06A1-4A4A-9B9C-CABB7A343CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8CE051-A18B-49E4-B627-B1F56A01DA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="156" yWindow="480" windowWidth="22884" windowHeight="10248" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="472">
   <si>
     <t>DAY 28 — MONETIZATION MODEL</t>
   </si>
@@ -1483,6 +1483,12 @@
   </si>
   <si>
     <t>Tôi tính tiền theo mỗi hóa đơn NCC được đối soát 3 chiều xong (theo định nghĩa job ở tab 1), giá 10.000 ₫/hóa đơn, với mức chi tiêu tối thiểu 1.000.000 ₫/tháng (tương đương 100 hóa đơn hoàn thành); khách điển hình 500 hóa đơn đầu vào có khoảng 160 hóa đơn hoàn thành nên trả theo lượt dùng, mức tối thiểu chỉ áp cho khách rất nhỏ.</t>
+  </si>
+  <si>
+    <t>Không áp dụng (Đã chọn đúng theo gợi ý của scorecard: USAGE)</t>
+  </si>
+  <si>
+    <t>Được</t>
   </si>
 </sst>
 </file>
@@ -6472,7 +6478,9 @@
       <c r="A31" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="B31" s="5"/>
+      <c r="B31" s="5" t="s">
+        <v>470</v>
+      </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
@@ -9157,25 +9165,33 @@
       <c r="A29" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="B29" s="5"/>
+      <c r="B29" s="5" t="s">
+        <v>471</v>
+      </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="B30" s="5"/>
+      <c r="B30" s="5" t="s">
+        <v>471</v>
+      </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="B31" s="5"/>
+      <c r="B31" s="5" t="s">
+        <v>471</v>
+      </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="B32" s="5"/>
+      <c r="B32" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>